<commit_message>
optimized visualization, the structure and standardizing the comments and output.
</commit_message>
<xml_diff>
--- a/results/master_summary.xlsx
+++ b/results/master_summary.xlsx
@@ -413,139 +413,279 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>评估维度与核心指标</t>
+          <t>Metric</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>模型输出数值</t>
+          <t>Value</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Q1 典型日最小购电费用 (元)</t>
+          <t>Q1 total purchase (kWh)</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>35126.95</v>
+        <v>59482.7</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Q1 典型日计划总购电量 (kWh)</t>
+          <t>Q1 total cost (Yuan)</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>59482.7</v>
+        <v>35126.95</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Q2 经验基准排产总成本 (元)</t>
+          <t>Q1 terminal SOC (kWh)</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>18832047.46</v>
+        <v>6000</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Q2 两阶段鲁棒优化总成本 (元)</t>
+          <t>Q2 baseline total cost (Yuan)</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>16085410.43</v>
+        <v>18832047.46</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Q2 相对基准方案节约费用 (元)</t>
+          <t>Q2 optimized total cost (Yuan)</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>2746637.03</v>
+        <v>16085410.43</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Q2 全年紧急购电总量 (kWh)</t>
+          <t>Q2 cost reduction (Yuan)</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>105491.12</v>
+        <v>2746637.03</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Q3 滚动时域 MPC 结算总成本 (元)</t>
+          <t>Q2 cost reduction (%)</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>15674191.15</v>
+        <v>14.58</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Q3 相对 Q2 调控避险节约 (元)</t>
+          <t>Q2 planned purchase (kWh)</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>411219.28</v>
+        <v>24764475.21</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Q3 全年紧急购电总量 (kWh)</t>
+          <t>Q2 emergency purchase (kWh)</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>49359.44</v>
+        <v>105491.12</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Q4-2 动态电价两阶段总成本 (元)</t>
+          <t>Q2 baseline Jan warm-up SOC (kWh)</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>16244576.3</v>
+        <v>10800</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Q4-3 动态电价滚动 MPC 总成本 (元)</t>
+          <t>Q2 optimized Jan warm-up SOC (kWh)</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>15810159.86</v>
+        <v>10723.37</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Q4 动态电价下 MPC 调控价值 (元)</t>
+          <t>Q3 planned purchase (kWh)</t>
         </is>
       </c>
       <c r="B13" t="n">
-        <v>434416.44</v>
+        <v>24856759.56</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Q3 adjusted purchase (kWh)</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>24267647.05</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Q3 emergency purchase (kWh)</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>52663.27</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Q3 total settlement cost (Yuan)</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>15808625.64</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Q3 saving vs Q2 (Yuan)</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>276784.79</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>Q3 saving vs Q2 (%)</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>1.72</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Q3 MPC fallback count</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Q4-2 total cost (Yuan)</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>16244576.3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Q4-2 emergency purchase (kWh)</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>109461.66</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Q4-3 total cost (Yuan)</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>15959374.62</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Q4-3 emergency purchase (kWh)</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>51420.02</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Q4-3 saving vs Q4-2 (Yuan)</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>285201.67</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Q4-3 saving vs Q4-2 (%)</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>1.76</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Q4 emergency reduction (%)</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>53.02</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Q4-3 MPC fallback count</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>